<commit_message>
Say in S6 that the fitness reference was exploratory, not a validation layer
The admissibility sheet described the Bloom and Neher estimates as reported in the main text.
The manuscript no longer reports the two medians it meant: the reference measures evolutionary
constraint rather than the quantity ranked here, and ranking its sites by effect magnitude
coincides with ranking them by constraint. The sheet now carries that status and the reason.

The analysis script, its result file and its pinned checksum are unchanged.
</commit_message>
<xml_diff>
--- a/supplementary/S6_Table.xlsx
+++ b/supplementary/S6_Table.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference matrix" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Layer admissibility" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Reference matrix" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Layer admissibility" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -5833,7 +5833,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
-    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="52" customWidth="1" min="2" max="2"/>
     <col width="52" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
@@ -6134,12 +6134,12 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>reported separately</t>
+          <t>exploratory characterization; not used for validation</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Measures evolutionary constraint rather than the quantity ranked here, so it characterizes the selected positions instead of scoring them. Reported in the main text for that reason.</t>
+          <t>Estimates evolutionary constraint from observed against expected counts, which is a different quantity from the one ranked here. Ranking its sites by effect magnitude coincides with ranking them by constraint, so the reference cannot separate whether a site has a measurable effect from whether it is constrained. Examined while candidate references were being surveyed and not used to validate the integrated score; the characterization it yields is written to results/functional_benchmark/fitness_characterisation.csv.</t>
         </is>
       </c>
     </row>

</xml_diff>